<commit_message>
Update layout, active navbar state, hover states, and remove mudec logo
</commit_message>
<xml_diff>
--- a/modello_progetti.xlsx
+++ b/modello_progetti.xlsx
@@ -1,42 +1,321 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/federicasilvestrini/Downloads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B59932-6B2E-2649-A855-120136A7A8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Progetti" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="74">
+  <si>
+    <t>Nome_Progetto</t>
+  </si>
+  <si>
+    <t>Immagine_Header</t>
+  </si>
+  <si>
+    <t>Titolo_Sottile_Intro</t>
+  </si>
+  <si>
+    <t>Titolo_Grassetto_Intro</t>
+  </si>
+  <si>
+    <t>Testo_Intro_Affianco_Al_Titolo</t>
+  </si>
+  <si>
+    <t>Titolo_Blocco_Testo_1</t>
+  </si>
+  <si>
+    <t>Testo_Blocco_1</t>
+  </si>
+  <si>
+    <t>Titolo_Blocco_Testo_2</t>
+  </si>
+  <si>
+    <t>Testo_Blocco_2</t>
+  </si>
+  <si>
+    <t>Immagini_Galleria</t>
+  </si>
+  <si>
+    <t>IL BULLONE</t>
+  </si>
+  <si>
+    <t>Fondazione</t>
+  </si>
+  <si>
+    <t>La penna come sibolo di rinascita</t>
+  </si>
+  <si>
+    <t>Per i giovani della Fondazione - i B.Livers - la scrittura è un atto catartico: raccontarsi diventa il primo passo per riconoscersi di nuovo come persone, e non solo come pazienti o ex-malati.
+La campagna mostra “gli effetti” che una penna può avere: alleggerire, far dimenticare la malattia e restituire la voglia di mettersi in gioco._x000B_Protagonisti sono cinque giovani redattori del giornale Il Bullone, che con le loro parole ci invitano a un gesto concreto: abbonarci o donare per permettere ad altri ragazzi di intraprendere lo stesso percorso.
+“Abbiamo scelto di raccontare la leggerezza ritrovata,” spiega Sergio Müller, Chief Communication Officer di A-Tono. “Cinque giovani e una penna, che diventa protagonista di piccoli momenti in cui si riscoprono come individui e non più solo come malati.</t>
+  </si>
+  <si>
+    <t>Una strategia digital-first per amplificare il valore</t>
+  </si>
+  <si>
+    <t>La campagna è stata pensata con un approccio digital-first, ottimizzando ogni euro investito per massimizzare impatto e conversione. La strategia media e i contenuti sono stati progettati per parlare alle persone giuste, nel modo più empatico, diretto e sostenibile possibile.
+“La collaborazione con A-Tono ETS ci permette di amplificare la voce dei nostri ragazzi e il valore del nostro modello,” afferma Bill Niada, fondatore e presidente di Fondazione Il Bullone. “Crediamo che questa campagna, potente nella sua autenticità e mirata nella strategia digital, ci aiuterà a raggiungere nuovi sostenitori indispensabili per garantire un futuro ai giovani che hanno affrontato esperienze di malattia grave.</t>
+  </si>
+  <si>
+    <t>Restituire valore alla società attraverso la comunicazione</t>
+  </si>
+  <si>
+    <t>Per A-Tono ETS, questo progetto è molto più di una campagna: è un modo per restituire valore alla società, mettendo creatività, competenza e tecnologia al servizio di chi costruisce futuro e speranza.
+“Siamo onorati di affiancare Fondazione Il Bullone in questa sfida,” racconta Anastasia Granato, presidentessa di A-Tono ETS. “Il Bullone non è solo un giornale, ma un vero laboratorio di rinascita. Il nostro obiettivo è stato tradurre la potenza emotiva di queste storie in una campagna digital efficace, capace di generare un impatto tangibile sulla vita dei B.Livers.”</t>
+  </si>
+  <si>
+    <t>bullone-1.jpg; bullone-2.jpg</t>
+  </si>
+  <si>
+    <t>Bullone</t>
+  </si>
+  <si>
+    <t>Partizan</t>
+  </si>
+  <si>
+    <t>A-Tono</t>
+  </si>
+  <si>
+    <t>A-Tono ETS è diventata anche una Società Sportiva, affiliata al C.S.I. – Centro Sportivo Italiano. Un passo naturale, per restituire, nel modo più concreto possibile, un po’ del nostro valore alla società.</t>
+  </si>
+  <si>
+    <t>Una squadra, tante storie</t>
+  </si>
+  <si>
+    <t>L’esordio vincente</t>
+  </si>
+  <si>
+    <t>Insieme al Partizan Bonola, associazione di quartiere attiva nel Municipio 8 di Milano, abbiamo messo in piedi una squadra di basket amatoriale per ragazzi tra i 18 e i 25 anni: A-Tono Partizan. Ragazzi con storie diverse, percorsi diversi, ma la stessa voglia di rimettersi in gioco.
+Usiamo lo sport per tenere lontane depressione, solitudine, ludopatia e avvicinare fiducia, vita di gruppo e salute.
+Perché un canestro a Bonola vale tre punti: promuove aggregazioni positive, restituisce possibilità, riqualifica un quartiere — proprio lì dove lo Stato arriva tardi.</t>
+  </si>
+  <si>
+    <t>L’esordio casalingo si è tenuto sabato 11 ottobre alle 19:30 al Palasoul di via Brivio 1 (Milano), con una vittoria che ha riempito di entusiasmo giocatori, staff e pubblico.
+Un risultato che va oltre il tabellone: è il segno di una comunità che cresce, che trova nello sport un linguaggio universale di energia, rispetto e rinascita.
+I ragazzi sono felici, grati, fieri.
+E noi con loro.</t>
+  </si>
+  <si>
+    <t>partizan-1.jpg partizan-2.jpg</t>
+  </si>
+  <si>
+    <t>MUDEC</t>
+  </si>
+  <si>
+    <t>MUDEC Gala</t>
+  </si>
+  <si>
+    <t>The Art of Giving</t>
+  </si>
+  <si>
+    <t>Non solo un evento, ma un vero e proprio manifesto.</t>
+  </si>
+  <si>
+    <t>Un nome che racconta l’essenza della serata, capace di intrecciare arte, alta cucina e tecnologia per sostenere cause ad alto impatto sociale. L’idea è semplice e trasformativa: unire arte, relazione e tecnologia per tradurre la bellezza in impatto sociale concreto e misurabile.
+Gli ospiti hanno vissuto un’esperienza fuori dall’ordinario: visita privata alla mostra M.C. Escher – L’arte e la scienza, seguita da una cena stellata firmata Enrico Bartolini, servita nell’Agorà del museo. 
+Il cuore della serata, però, non era nel programma, bensì nei due progetti presentati da Anastasia Granato, presidentessa di A-Tono ETS. Da un lato, la campagna abbonamenti “Un Bullone per rinascere” rivolta alle aziende per Il Bullone, il giornale che accompagna giovani colpiti da malattie oncologiche o autoimmuni in un percorso di rinascita attraverso la scrittura; dall’altro, un’installazione pubblica, “La Cabina Rosa”, dedicata alla prevenzione e al riconoscimento della violenza di genere, con un’azione di sensibilizzazione che promuove il 1522, numero nazionale antiviolenza e stalking.
+Come ha ricordato la presidentessa Anastasia Granato, il dono è “arte delle connessioni”: tra tasselli diversi - persone, competenze, organizzazioni - che, accostati con cura, compongono un’immagine più grande. 
+A rendere “The Art of Giving” un modello unico nel suo genere è stata anche la tecnologia: sui tavoli infatti, i DropPOS A-Tono (terminali di pagamento contactless sviluppati dal gruppo) hanno permesso donazioni aggiuntive immediate, semplici e sicure, trasformando l’atto del donare in un processo più accessibile, naturale e diffuso.</t>
+  </si>
+  <si>
+    <t>partizan-header.jpg</t>
+  </si>
+  <si>
+    <t>mudec-header.jpg</t>
+  </si>
+  <si>
+    <t>bullone-header.jpg</t>
+  </si>
+  <si>
+    <t>mudec-1.jpg</t>
+  </si>
+  <si>
+    <t>Cabina Rosa</t>
+  </si>
+  <si>
+    <t>Installazione urbana</t>
+  </si>
+  <si>
+    <t>La Cabina Rosa di A-Tono ETS: il giorno in cui Milano si è fermata ad ascoltare</t>
+  </si>
+  <si>
+    <t>In occasione della Giornata internazionale per l’eliminazione della violenza contro le donne, il 25 novembre, in CityLife a Milano è successo qualcosa di raro: la città, per qualche ora, ha rallentato.
+In Piazza Tre Torri, la Cabina Rosa a sostegno del numero antiviolenza e antistalking 1522 ha richiamato centinaia di persone, guidate da una spettacolare domination degli schermi Mediamond che, come un filo luminoso, accompagnava i passanti fino all’installazione.
+La cabina, una presenza d’altri tempi nel quartiere più contemporaneo di Milano, si è riempita senza sosta. Passanti, studenti, volontari, creator: ognuno entrava, ascoltava, usciva diverso. Dentro, i messaggi arrivavano con delicatezza: brevi dialoghi che raccontano la violenza tra le righe; quella che sfugge a tanti fino a quando quella violenza diventa reale, e ci si trova a ripetere “potevamo accorgerci prima”.</t>
+  </si>
+  <si>
+    <t>“La violenza, spesso, si racconta solo a metà. Serve qualcuno che ascolti, dall’altra parte, chiunque esso sia”, ha ricordato Anastasia Granato, presidentessa di A-Tono ETS. “Prestare attenzione può veramente cambiare le cose, prima che sia troppo tardi”.
+Ed è esattamente quello che la giornata di ieri ha dimostrato: l’ascolto, quando accade, trasforma le persone e, speriamo, le cose.</t>
+  </si>
+  <si>
+    <t>Il percorso che ha portato fin qui</t>
+  </si>
+  <si>
+    <t>La Cabina Rosa è l’ultimo passo di un progetto che si è sviluppato in tre momenti:
+Il silenzio che squilla.
+Un video teaser ha mostrato telefoni rossi che suonano in mezzo alla folla. Nessuno rispondeva, finché una voce, quella di un’operatrice del 1522, rompeva il buio dello schermo. Un invito chiaro: scegliere di agire.
+Passala.
+Poi è arrivato il coinvolgimento dei creator, ognuno con una cornetta rossa da collegare al telefono: un simbolo potente, quasi fisico, che li invitava a parlare, ascoltare, intervenire. E ieri molti di loro erano lì, a “passare la cornetta” anche offline.
+Cabina Rosa: l’installazione urbana.
+Dal 22 al 29 novembre la cabina rimarrà in Piazza Tre Torri, accanto a pannelli informativi che mostrano come riconoscere i segnali nascosti della violenza e come poter aiutare.
+“Abbiamo scelto il linguaggio più immediato che esista: una chiamata. Ascoltarla è la prima azione che invitiamo a compiere”. ha spiegato Sergio Müller, Chief Communication Officer di A-Tono.
+Un gesto semplice, quasi istintivo, eppure capace di aprire conversazioni profonde e forse cambiare le cose.
+Una comunità che risponde
+La piazza è diventata un punto di incontro spontaneo: chi ascoltava, chi faceva domande, chi restava a leggere, chi rientrava per capire meglio.
+Un movimento silenzioso, fatto di piccoli gesti che insieme hanno creato una comunità temporanea.
+“CityLife è un luogo che vive del dialogo tra persone, spazi e idee”, ha dichiarato Roberto Russo, Amministratore Delegato di SmartCityLife. “Siamo orgogliosi di ospitare un progetto che invita la città a fermarsi, ad ascoltare e a rispondere”.
+È esattamente quello che è accaduto.
+Grazie. Di cuore.
+Grazie a chi è entrato nella Cabina Rosa.
+A chi ha ascoltato fino in fondo.
+Ai volontari, ai creator, ai passanti diventati partecipanti.
+E grazie a CityLife per l’accoglienza, a Mediamond per una visibilità che ha amplificato il messaggio in tutto il quartiere, e al Comune di Milano e alla Regione Lombardia per i patrocini che sostengono una causa che riguarda tutti.</t>
+  </si>
+  <si>
+    <t>cabina-header.jpg</t>
+  </si>
+  <si>
+    <t>cabina-1.jpg</t>
+  </si>
+  <si>
+    <t>Restart Romagna</t>
+  </si>
+  <si>
+    <t>Campagna</t>
+  </si>
+  <si>
+    <t>Re-start Romagna</t>
+  </si>
+  <si>
+    <t>DropTicket solidale: donati 5000 Euro alla Protezione Civile grazie alla Campagna "Re-Start Romagna"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In seguito all’alluvione che ha colpito la Romagna in maggio, abbiamo deciso di mettere in atto un'iniziativa unica per aiutare la regione a risollevarsi dagli effetti della catastrofe.
+Come? “Hackerando” la nostra piattaforma di biglietteria DropTicket in modo creativo, per raccogliere fondi destinati alla Protezione Civile dell'Emilia Romagna, permettendo ai nostri utenti di farlo con la stessa facilità con cui avrebbero acquistato un biglietto.
+Abbiamo creato un biglietto virtuale che non avrebbe fatto viaggiare le persone, ma la loro solidarietà, e lo abbiamo chiamato "Re-Start Romagna". 
+È stato comunicato attraverso il sito, l’app, dem agli utenti e sui canali social.
+Le entrate generate dalla vendita di questi biglietti virtuali sarebbero state interamente devolute alla Protezione Civile, per supportare le operazioni di soccorso e ripristino in seguito all'alluvione.
+Nelle scorse settimane è stata completata con successo la raccolta fondi ed è stato emesso un trasferimento bancario di 5000 euro destinati alla Protezione Civile dell'Emilia Romagna. Questa donazione rappresenta il risultato tangibile dell'impegno e della partecipazione delle persone alla campagna "Re-Start Romagna".
+La risposta della comunità è stata straordinaria, dimostrando ancora una volta quanto possa essere potente l'uso della tecnologia e della solidarietà congiunte. </t>
+  </si>
+  <si>
+    <t>Scopri la case sul progetto qui:</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zkXhsGLq2-c&amp;t=1s</t>
+  </si>
+  <si>
+    <t>restart-header.jpg</t>
+  </si>
+  <si>
+    <t>Non esistono ragazzi cattivi</t>
+  </si>
+  <si>
+    <t>Un percorso di rebranding che unisce strategia, creatività e comunicazione per dare maggiore forza e riconoscibilità alla realtà di Kayros.</t>
+  </si>
+  <si>
+    <t>Kayros – Un’identità che racconta una seconda possibilità</t>
+  </si>
+  <si>
+    <t>Per Kayros – Non esistono ragazzi cattivi – abbiamo sviluppato un progetto di rebranding e di declinazione dell'identità visiva, con l'obiettivo di valorizzare una realtà che ogni giorno accompagna adolescenti e giovani adulti in percorsi di crescita, inclusione e riscatto attraverso attività educative, artistiche e musicali. La comunità offre infatti opportunità concrete di reinserimento sociale, facendo della musica uno dei principali strumenti di espressione e rinascita.
+Il progetto è partito dal restyling del logo, studiato per rappresentare in modo più contemporaneo e riconoscibile i valori di accoglienza, speranza e cambiamento che contraddistinguono Kayros. Da questa nuova identità è nato un sistema visivo coerente, capace di adattarsi ai diversi punti di contatto dell'associazione e di rafforzarne la presenza sul territorio.
+Abbiamo inoltre progettato una linea di merchandising coordinato, pensata non solo come strumento di comunicazione, ma anche come elemento in grado di trasmettere il senso di appartenenza alla comunità e di diffondere il messaggio positivo dell'associazione.
+Il lavoro è stato completato con una serie di proposte per l'allestimento degli spazi della sede e lo sviluppo grafico di ulteriori supporti fisici e istituzionali. Ogni concept è stato realizzato con l'obiettivo di creare un'identità forte, riconoscibile e facilmente declinabile, capace di accompagnare Kayros nelle sue attività quotidiane e negli eventi pubblici, contribuendo a raccontare con coerenza una realtà che crede nel valore delle persone e nella possibilità di offrire a ogni ragazzo una nuova occasione.</t>
+  </si>
+  <si>
+    <t>kayros-header.jpg</t>
+  </si>
+  <si>
+    <t>kayros-1.jpg; kayros-2.jpg</t>
+  </si>
+  <si>
+    <t>Un Cuore Un Mondo</t>
+  </si>
+  <si>
+    <t>Un Cuore</t>
+  </si>
+  <si>
+    <t>Un Mondo</t>
+  </si>
+  <si>
+    <t>Un progetto di rebranding e comunicazione sociale nato per dare maggiore visibilità all'associazione e sensibilizzare il pubblico sulle cardiopatie congenite pediatriche.</t>
+  </si>
+  <si>
+    <t>Un Cuore Un Mondo – Quando un errore diventa un messaggio</t>
+  </si>
+  <si>
+    <t>Per Un Cuore Un Mondo Massa abbiamo sviluppato un percorso di rinnovamento della brand identity, partendo dal restyling del logo e dalla definizione di una nuova immagine coordinata, capace di rappresentare con maggiore forza la missione dell'associazione: sostenere il reparto di cardiochirurgia pediatrica dell'Ospedale del Cuore di Massa e le famiglie dei piccoli pazienti.
+Abbiamo inoltre ideato e realizzato la campagna "Mettiamoci il Quore", un concept creativo costruito attorno alla parola quore: un cuore con un piccolo o grande "errore", simbolo delle cardiopatie congenite. Attraverso questo gioco linguistico abbiamo creato contenuti social, copy e attivazioni dedicate, invitando le persone a partecipare alla #SfidaDelQuore e a diffondere un messaggio di vicinanza, consapevolezza e sostegno.
+Negli anni la collaborazione si è estesa anche allo sviluppo di strumenti operativi e materiali di supporto, tra cui un database gestionale, attività di sponsorizzazione, forniture e ulteriori iniziative di comunicazione. Un progetto costruito nel tempo per contribuire, con creatività e competenze, a una causa che mette ogni giorno al centro il benessere dei bambini e delle loro famiglie.</t>
+  </si>
+  <si>
+    <t>cuoremondo-1.jpg</t>
+  </si>
+  <si>
+    <t>cuoremondo-header.jpg</t>
+  </si>
+  <si>
+    <t>PARTIZAN</t>
+  </si>
+  <si>
+    <t>CABINA ROSA</t>
+  </si>
+  <si>
+    <t>Kayros</t>
+  </si>
+  <si>
+    <t>KAYROS</t>
+  </si>
+  <si>
+    <t>Ci sono progetti che ci ricordano perché facciamo questo mestiere. Collaborare con Fondazione Il Bullone è uno di questi. Con loro abbiamo ideato e lanciato la nuova campagna digital di raccolta fondi individui della Fondazione. Un progetto che parla di rinascita, coraggio e comunicazione come strumento di cambiamento reale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venerdì 3 ottobre 2025, nella cornice del MUDEC - Museo delle Culture di Milano, A-Tono ETS ha firmato il suo debutto pubblico con il Gala “The Art of Giving”. </t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -64,14 +343,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,88 +687,486 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18.1640625" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="4" max="4" width="22.5" customWidth="1"/>
+    <col min="5" max="5" width="31.33203125" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+    <col min="7" max="9" width="19.1640625" customWidth="1"/>
+    <col min="10" max="10" width="21.6640625" customWidth="1"/>
+    <col min="11" max="11" width="24.6640625" customWidth="1"/>
+    <col min="12" max="12" width="31" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Nome_Progetto</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Immagine_Header</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Logo_Sinistra</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Logo_Destra</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Titolo_Sottile_Intro</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Titolo_Grassetto_Intro</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Testo_Intro_Affianco_Al_Titolo</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Titolo_Blocco_Testo_1</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Testo_Blocco_1</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Titolo_Blocco_Testo_2</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Testo_Blocco_2</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Immagini_Galleria</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Il Bullone Esempio</v>
-      </c>
-      <c r="B2" t="str">
-        <v>header-bullone.jpg</v>
-      </c>
-      <c r="C2" t="str">
-        <v>logo-bullone.png</v>
-      </c>
-      <c r="D2" t="str">
-        <v>logo-ets.png</v>
-      </c>
-      <c r="E2" t="str">
-        <v>progetto di giornalismo</v>
-      </c>
-      <c r="F2" t="str">
-        <v>IL BULLONE</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Questo è il testo che andrà a destra della linea e del titolo introduttivo.</v>
-      </c>
-      <c r="H2" t="str">
-        <v>L'INIZIATIVA</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Questo è il primo blocco di testo principale che andrà sotto a tutta larghezza.</v>
-      </c>
-      <c r="J2" t="str">
-        <v>I RISULTATI</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Questo è un secondo blocco di testo facoltativo. Puoi lasciarlo vuoto.</v>
-      </c>
-      <c r="L2" t="str">
-        <v>foto1.jpg, foto2.jpg, foto3.jpg</v>
-      </c>
+    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="2" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError sqref="A1:B1 D3 D1:G1 L1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>